<commit_message>
Daily slate 2026-06-23 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-21.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-21.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E2" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F2" t="n">
         <v>126</v>
       </c>
       <c r="G2" t="n">
-        <v>46.8</v>
+        <v>47.3</v>
       </c>
     </row>
     <row r="3">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="E4" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F4" t="n">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="G4" t="n">
-        <v>29.6</v>
+        <v>29.4</v>
       </c>
     </row>
     <row r="5">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E7" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G7" t="n">
-        <v>48.6</v>
+        <v>49.1</v>
       </c>
     </row>
     <row r="8">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E9" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F9" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G9" t="n">
-        <v>45.9</v>
+        <v>46.2</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1056</v>
+        <v>1133</v>
       </c>
       <c r="E11" t="n">
-        <v>657</v>
+        <v>702</v>
       </c>
       <c r="F11" t="n">
-        <v>399</v>
+        <v>431</v>
       </c>
       <c r="G11" t="n">
-        <v>62.2</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E12" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F12" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G12" t="n">
-        <v>64.09999999999999</v>
+        <v>63.9</v>
       </c>
     </row>
     <row r="13">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="E14" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F14" t="n">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="G14" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>513</v>
+        <v>521</v>
       </c>
       <c r="E15" t="n">
         <v>93</v>
       </c>
       <c r="F15" t="n">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="G15" t="n">
-        <v>18.1</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="E16" t="n">
         <v>56</v>
       </c>
       <c r="F16" t="n">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="G16" t="n">
-        <v>19.7</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5220</v>
+        <v>5554</v>
       </c>
       <c r="E17" t="n">
-        <v>935</v>
+        <v>980</v>
       </c>
       <c r="F17" t="n">
-        <v>4285</v>
+        <v>4574</v>
       </c>
       <c r="G17" t="n">
-        <v>17.9</v>
+        <v>17.6</v>
       </c>
     </row>
   </sheetData>
@@ -1582,16 +1582,16 @@
         <v>373</v>
       </c>
       <c r="D7" t="n">
-        <v>62.2</v>
+        <v>62</v>
       </c>
       <c r="E7" t="n">
-        <v>1056</v>
+        <v>1133</v>
       </c>
       <c r="F7" t="n">
-        <v>64.09999999999999</v>
+        <v>63.9</v>
       </c>
       <c r="G7" t="n">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H7" t="n">
         <v>54.3</v>
@@ -1600,40 +1600,40 @@
         <v>105</v>
       </c>
       <c r="J7" t="n">
-        <v>24.5</v>
+        <v>24.7</v>
       </c>
       <c r="K7" t="n">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="L7" t="n">
-        <v>18.1</v>
+        <v>17.9</v>
       </c>
       <c r="M7" t="n">
-        <v>513</v>
+        <v>521</v>
       </c>
       <c r="N7" t="n">
-        <v>19.7</v>
+        <v>19.5</v>
       </c>
       <c r="O7" t="n">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="P7" t="n">
-        <v>17.9</v>
+        <v>17.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>5220</v>
+        <v>5554</v>
       </c>
       <c r="R7" t="n">
-        <v>46.8</v>
+        <v>47.3</v>
       </c>
       <c r="S7" t="n">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="T7" t="n">
-        <v>29.6</v>
+        <v>29.4</v>
       </c>
       <c r="U7" t="n">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
@@ -1660,16 +1660,16 @@
         <v>21</v>
       </c>
       <c r="AD7" t="n">
-        <v>48.6</v>
+        <v>49.1</v>
       </c>
       <c r="AE7" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="AF7" t="n">
-        <v>45.9</v>
+        <v>46.2</v>
       </c>
       <c r="AG7" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>